<commit_message>
Suppression de la contrainte de card minimale de relatesTo
Suite à la demande de @aperie07 25c073960083444ccd7dba2b64d82cee9c1f9968
</commit_message>
<xml_diff>
--- a/nriss-patch-2/ig/StructureDefinition-fr-allergy-intolerance-document.xlsx
+++ b/nriss-patch-2/ig/StructureDefinition-fr-allergy-intolerance-document.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AM$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AM$49</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1466" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1741" uniqueCount="385">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-04T07:44:41+00:00</t>
+    <t>2026-08-07T09:15:45+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -555,25 +555,155 @@
 Class</t>
   </si>
   <si>
+    <t>allergy | intolerance - Underlying mechanism (if known)</t>
+  </si>
+  <si>
+    <t>Identification of the underlying physiological mechanism for the reaction risk.</t>
+  </si>
+  <si>
+    <t>Allergic (typically immune-mediated) reactions have been traditionally regarded as an indicator for potential escalation to significant future risk. Contemporary knowledge suggests that some reactions previously thought to be immune-mediated are, in fact, non-immune, but in some cases can still pose a life threatening risk. It is acknowledged that many clinicians might not be in a position to distinguish the mechanism of a particular reaction. Often the term "allergy" is used rather generically and may overlap with the use of "intolerance" - in practice the boundaries between these two concepts might not be well-defined or understood. This data element is included nevertheless, because many legacy systems have captured this attribute. Immunologic testing may provide supporting evidence for the basis of the reaction and the causative substance, but no tests are 100% sensitive or specific for sensitivity to a particular substance. If, as is commonly the case, it is unclear whether the reaction is due to an allergy or an intolerance, then the type element should be omitted from the resource.</t>
+  </si>
+  <si>
+    <t>Identification of the underlying physiological mechanism for a Reaction Risk.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/allergy-intolerance-type|4.0.1</t>
+  </si>
+  <si>
+    <t>code</t>
+  </si>
+  <si>
+    <t>FiveWs.class</t>
+  </si>
+  <si>
+    <t>IAM-9</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">string
+</t>
+  </si>
+  <si>
+    <t>xml:id (or equivalent in JSON)</t>
+  </si>
+  <si>
+    <t>unique id for the element within a resource (for internal references)</t>
+  </si>
+  <si>
+    <t>Element.id</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension</t>
+  </si>
+  <si>
+    <t>Extension</t>
+  </si>
+  <si>
+    <t>An Extension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value:url}
+</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>Element.extension</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension:type</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {http://hl7.org/fhir/5.0/StructureDefinition/extension-AllergyIntolerance.type|0.1.0}
+</t>
+  </si>
+  <si>
     <t>Type d'allergie ou d'intolérance</t>
   </si>
   <si>
-    <t>Identification of the underlying physiological mechanism for the reaction risk.</t>
-  </si>
-  <si>
-    <t>Allergic (typically immune-mediated) reactions have been traditionally regarded as an indicator for potential escalation to significant future risk. Contemporary knowledge suggests that some reactions previously thought to be immune-mediated are, in fact, non-immune, but in some cases can still pose a life threatening risk. It is acknowledged that many clinicians might not be in a position to distinguish the mechanism of a particular reaction. Often the term "allergy" is used rather generically and may overlap with the use of "intolerance" - in practice the boundaries between these two concepts might not be well-defined or understood. This data element is included nevertheless, because many legacy systems have captured this attribute. Immunologic testing may provide supporting evidence for the basis of the reaction and the causative substance, but no tests are 100% sensitive or specific for sensitivity to a particular substance. If, as is commonly the case, it is unclear whether the reaction is due to an allergy or an intolerance, then the type element should be omitted from the resource.</t>
+    <t>R5: `AllergyIntolerance.type` additional types (CodeableConcept) additional types from child elements (coding)</t>
+  </si>
+  <si>
+    <t>Element `AllergyIntolerance.type` is mapped to FHIR R4 element `AllergyIntolerance.type` as `SourceIsBroaderThanTarget`.
+The mappings for `AllergyIntolerance.type` do not cover the following types: CodeableConcept.
+The mappings for `AllergyIntolerance.type` do not cover the following types based on type expansion: coding.
+Allergic (typically immune-mediated) reactions have been traditionally regarded as an indicator for potential escalation to significant future risk. Contemporary knowledge suggests that some reactions previously thought to be immune-mediated are, in fact, non-immune, but in some cases can still pose a life threatening risk. It is acknowledged that many clinicians might not be in a position to distinguish the mechanism of a particular reaction. Often the term "allergy" is used rather generically and may overlap with the use of "intolerance" - in practice the boundaries between these two concepts might not be well-defined or understood. This data element is included nevertheless, because many legacy systems have captured this attribute. Immunologic testing may provide supporting evidence for the basis of the reaction and the causative substance, but no tests are 100% sensitive or specific for sensitivity to a particular substance. If, as is commonly the case, it is unclear whether the reaction is due to an allergy or an intolerance, then the type element should be omitted from the resource.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ele-1
+</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension:type.id</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension.id</t>
+  </si>
+  <si>
+    <t>Unique id for inter-element referencing</t>
+  </si>
+  <si>
+    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension:type.extension</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension.extension</t>
+  </si>
+  <si>
+    <t>Extensions are always sliced by (at least) url</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension:type.url</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension.url</t>
+  </si>
+  <si>
+    <t>identifies the meaning of the extension</t>
+  </si>
+  <si>
+    <t>Source of the definition for the extension code - a logical name or a URL.</t>
+  </si>
+  <si>
+    <t>The definition may point directly to a computable or human-readable definition of the extensibility codes, or it may be a logical URI as declared in some other specification. The definition SHALL be a URI for the Structure Definition defining the extension.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/5.0/StructureDefinition/extension-AllergyIntolerance.type</t>
+  </si>
+  <si>
+    <t>Extension.url</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension:type.value[x]</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.extension.value[x]</t>
   </si>
   <si>
     <t>https://interop.esante.gouv.fr/ig/fhir/document-core/ValueSet/fr-vs-allergy-intolerance-type-document|0.1.0</t>
   </si>
   <si>
-    <t>code</t>
-  </si>
-  <si>
-    <t>FiveWs.class</t>
-  </si>
-  <si>
-    <t>IAM-9</t>
+    <t>Extension.value[x]</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.type.value</t>
+  </si>
+  <si>
+    <t>Primitive value for code</t>
+  </si>
+  <si>
+    <t>string.value</t>
   </si>
   <si>
     <t>AllergyIntolerance.category</t>
@@ -742,9 +872,6 @@
 </t>
   </si>
   <si>
-    <t>open</t>
-  </si>
-  <si>
     <t>effectiveTime.low</t>
   </si>
   <si>
@@ -770,22 +897,6 @@
     <t>AllergyIntolerance.onset[x].id</t>
   </si>
   <si>
-    <t xml:space="preserve">string
-</t>
-  </si>
-  <si>
-    <t>Unique id for inter-element referencing</t>
-  </si>
-  <si>
-    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
-  </si>
-  <si>
-    <t>Element.id</t>
-  </si>
-  <si>
-    <t>n/a</t>
-  </si>
-  <si>
     <t>AllergyIntolerance.onset[x]:onsetPeriod.extension</t>
   </si>
   <si>
@@ -793,16 +904,6 @@
   </si>
   <si>
     <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value:url}
-</t>
-  </si>
-  <si>
-    <t>Extensions are always sliced by (at least) url</t>
-  </si>
-  <si>
-    <t>Element.extension</t>
   </si>
   <si>
     <t>AllergyIntolerance.onset[x]:onsetPeriod.start</t>
@@ -1449,7 +1550,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AM41"/>
+  <dimension ref="A1:AM49"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="40.31640625" customWidth="true" bestFit="true"/>
@@ -3010,9 +3111,11 @@
       <c r="X14" t="s" s="2">
         <v>158</v>
       </c>
-      <c r="Y14" s="2"/>
+      <c r="Y14" t="s" s="2">
+        <v>175</v>
+      </c>
       <c r="Z14" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AA14" t="s" s="2">
         <v>79</v>
@@ -3045,32 +3148,32 @@
         <v>99</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AL14" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AM14" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
-        <v>180</v>
+        <v>79</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G15" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H15" t="s" s="2">
         <v>79</v>
@@ -3079,20 +3182,18 @@
         <v>79</v>
       </c>
       <c r="J15" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>107</v>
+        <v>181</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>182</v>
-      </c>
-      <c r="N15" t="s" s="2">
         <v>183</v>
       </c>
+      <c r="N15" s="2"/>
       <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">
         <v>79</v>
@@ -3117,93 +3218,91 @@
         <v>79</v>
       </c>
       <c r="X15" t="s" s="2">
-        <v>158</v>
+        <v>79</v>
       </c>
       <c r="Y15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF15" t="s" s="2">
         <v>184</v>
       </c>
-      <c r="Z15" t="s" s="2">
+      <c r="AG15" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH15" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AK15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AL15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM15" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16" hidden="true">
+      <c r="A16" t="s" s="2">
         <v>185</v>
       </c>
-      <c r="AA15" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB15" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC15" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD15" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE15" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF15" t="s" s="2">
-        <v>179</v>
-      </c>
-      <c r="AG15" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH15" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AI15" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AJ15" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AK15" t="s" s="2">
-        <v>186</v>
-      </c>
-      <c r="AL15" t="s" s="2">
-        <v>177</v>
-      </c>
-      <c r="AM15" t="s" s="2">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s" s="2">
-        <v>188</v>
-      </c>
       <c r="B16" t="s" s="2">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
-        <v>189</v>
+        <v>79</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G16" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H16" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="I16" t="s" s="2">
         <v>79</v>
       </c>
       <c r="J16" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>107</v>
+        <v>133</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>191</v>
-      </c>
-      <c r="N16" t="s" s="2">
-        <v>192</v>
-      </c>
+        <v>187</v>
+      </c>
+      <c r="N16" s="2"/>
       <c r="O16" s="2"/>
       <c r="P16" t="s" s="2">
         <v>79</v>
@@ -3228,92 +3327,92 @@
         <v>79</v>
       </c>
       <c r="X16" t="s" s="2">
-        <v>158</v>
+        <v>79</v>
       </c>
       <c r="Y16" t="s" s="2">
-        <v>193</v>
+        <v>79</v>
       </c>
       <c r="Z16" t="s" s="2">
-        <v>194</v>
+        <v>79</v>
       </c>
       <c r="AA16" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AB16" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC16" t="s" s="2">
-        <v>79</v>
-      </c>
+        <v>188</v>
+      </c>
+      <c r="AC16" s="2"/>
       <c r="AD16" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE16" t="s" s="2">
-        <v>79</v>
+        <v>189</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH16" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI16" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ16" t="s" s="2">
-        <v>99</v>
+        <v>138</v>
       </c>
       <c r="AK16" t="s" s="2">
-        <v>195</v>
+        <v>79</v>
       </c>
       <c r="AL16" t="s" s="2">
-        <v>196</v>
+        <v>79</v>
       </c>
       <c r="AM16" t="s" s="2">
-        <v>197</v>
+        <v>79</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>198</v>
-      </c>
-      <c r="C17" s="2"/>
+        <v>185</v>
+      </c>
+      <c r="C17" t="s" s="2">
+        <v>192</v>
+      </c>
       <c r="D17" t="s" s="2">
-        <v>199</v>
+        <v>79</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" t="s" s="2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="G17" t="s" s="2">
         <v>87</v>
       </c>
       <c r="H17" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="I17" t="s" s="2">
         <v>79</v>
       </c>
       <c r="J17" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>154</v>
+        <v>193</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="N17" t="s" s="2">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
@@ -3339,11 +3438,13 @@
         <v>79</v>
       </c>
       <c r="X17" t="s" s="2">
-        <v>203</v>
-      </c>
-      <c r="Y17" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="Y17" t="s" s="2">
+        <v>79</v>
+      </c>
       <c r="Z17" t="s" s="2">
-        <v>204</v>
+        <v>79</v>
       </c>
       <c r="AA17" t="s" s="2">
         <v>79</v>
@@ -3361,65 +3462,65 @@
         <v>79</v>
       </c>
       <c r="AF17" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="AG17" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH17" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI17" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="AJ17" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="AK17" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AL17" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM17" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" hidden="true">
+      <c r="A18" t="s" s="2">
         <v>198</v>
       </c>
-      <c r="AG17" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH17" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI17" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AJ17" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AK17" t="s" s="2">
-        <v>205</v>
-      </c>
-      <c r="AL17" t="s" s="2">
-        <v>206</v>
-      </c>
-      <c r="AM17" t="s" s="2">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s" s="2">
-        <v>208</v>
-      </c>
       <c r="B18" t="s" s="2">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>209</v>
+        <v>79</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="G18" t="s" s="2">
         <v>87</v>
       </c>
       <c r="H18" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="I18" t="s" s="2">
         <v>79</v>
       </c>
       <c r="J18" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>210</v>
+        <v>181</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -3470,10 +3571,10 @@
         <v>79</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>208</v>
+        <v>184</v>
       </c>
       <c r="AG18" t="s" s="2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="AH18" t="s" s="2">
         <v>87</v>
@@ -3482,24 +3583,24 @@
         <v>79</v>
       </c>
       <c r="AJ18" t="s" s="2">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="AK18" t="s" s="2">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>214</v>
+        <v>79</v>
       </c>
       <c r="AM18" t="s" s="2">
-        <v>215</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>216</v>
+        <v>203</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3510,7 +3611,7 @@
         <v>77</v>
       </c>
       <c r="G19" t="s" s="2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="H19" t="s" s="2">
         <v>79</v>
@@ -3522,13 +3623,13 @@
         <v>79</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>217</v>
+        <v>133</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>218</v>
+        <v>186</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>219</v>
+        <v>187</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -3567,37 +3668,37 @@
         <v>79</v>
       </c>
       <c r="AB19" t="s" s="2">
-        <v>79</v>
+        <v>188</v>
       </c>
       <c r="AC19" t="s" s="2">
-        <v>79</v>
+        <v>205</v>
       </c>
       <c r="AD19" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE19" t="s" s="2">
-        <v>79</v>
+        <v>189</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>216</v>
+        <v>190</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH19" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI19" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>99</v>
+        <v>138</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>220</v>
+        <v>79</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>221</v>
+        <v>79</v>
       </c>
       <c r="AM19" t="s" s="2">
         <v>79</v>
@@ -3605,10 +3706,10 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>222</v>
+        <v>206</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>222</v>
+        <v>207</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -3616,13 +3717,13 @@
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G20" t="s" s="2">
         <v>87</v>
       </c>
       <c r="H20" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="I20" t="s" s="2">
         <v>79</v>
@@ -3631,22 +3732,24 @@
         <v>79</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>223</v>
+        <v>101</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>224</v>
+        <v>208</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>225</v>
-      </c>
-      <c r="N20" s="2"/>
+        <v>209</v>
+      </c>
+      <c r="N20" t="s" s="2">
+        <v>210</v>
+      </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
         <v>79</v>
       </c>
       <c r="Q20" s="2"/>
       <c r="R20" t="s" s="2">
-        <v>79</v>
+        <v>211</v>
       </c>
       <c r="S20" t="s" s="2">
         <v>79</v>
@@ -3676,20 +3779,22 @@
         <v>79</v>
       </c>
       <c r="AB20" t="s" s="2">
-        <v>226</v>
-      </c>
-      <c r="AC20" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="AC20" t="s" s="2">
+        <v>79</v>
+      </c>
       <c r="AD20" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE20" t="s" s="2">
-        <v>227</v>
+        <v>79</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="AG20" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="AH20" t="s" s="2">
         <v>87</v>
@@ -3698,28 +3803,26 @@
         <v>79</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>228</v>
+        <v>130</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>229</v>
+        <v>79</v>
       </c>
       <c r="AM20" t="s" s="2">
         <v>79</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>230</v>
+        <v>213</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="C21" t="s" s="2">
-        <v>231</v>
-      </c>
+        <v>214</v>
+      </c>
+      <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
         <v>79</v>
       </c>
@@ -3731,7 +3834,7 @@
         <v>87</v>
       </c>
       <c r="H21" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="I21" t="s" s="2">
         <v>79</v>
@@ -3740,15 +3843,17 @@
         <v>79</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>232</v>
+        <v>154</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>233</v>
+        <v>172</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>225</v>
-      </c>
-      <c r="N21" s="2"/>
+        <v>173</v>
+      </c>
+      <c r="N21" t="s" s="2">
+        <v>174</v>
+      </c>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
         <v>79</v>
@@ -3773,13 +3878,11 @@
         <v>79</v>
       </c>
       <c r="X21" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y21" t="s" s="2">
-        <v>79</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="Y21" s="2"/>
       <c r="Z21" t="s" s="2">
-        <v>79</v>
+        <v>215</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>79</v>
@@ -3797,7 +3900,7 @@
         <v>79</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>77</v>
@@ -3812,10 +3915,10 @@
         <v>99</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>228</v>
+        <v>130</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>229</v>
+        <v>79</v>
       </c>
       <c r="AM21" t="s" s="2">
         <v>79</v>
@@ -3823,10 +3926,10 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>234</v>
+        <v>217</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>235</v>
+        <v>217</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3849,13 +3952,13 @@
         <v>79</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>236</v>
+        <v>181</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>237</v>
+        <v>218</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>238</v>
+        <v>218</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3906,7 +4009,7 @@
         <v>79</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>239</v>
+        <v>219</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>77</v>
@@ -3921,7 +4024,7 @@
         <v>79</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>240</v>
+        <v>79</v>
       </c>
       <c r="AL22" t="s" s="2">
         <v>79</v>
@@ -3932,14 +4035,14 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>241</v>
+        <v>220</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>242</v>
+        <v>220</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>132</v>
+        <v>221</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
@@ -3955,19 +4058,19 @@
         <v>79</v>
       </c>
       <c r="J23" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>134</v>
+        <v>222</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>136</v>
+        <v>224</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -3993,31 +4096,31 @@
         <v>79</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>79</v>
+        <v>158</v>
       </c>
       <c r="Y23" t="s" s="2">
-        <v>79</v>
+        <v>225</v>
       </c>
       <c r="Z23" t="s" s="2">
-        <v>79</v>
+        <v>226</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AB23" t="s" s="2">
-        <v>244</v>
+        <v>79</v>
       </c>
       <c r="AC23" t="s" s="2">
-        <v>245</v>
+        <v>79</v>
       </c>
       <c r="AD23" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE23" t="s" s="2">
-        <v>227</v>
+        <v>79</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>246</v>
+        <v>220</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>77</v>
@@ -4029,38 +4132,38 @@
         <v>79</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>138</v>
+        <v>99</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>240</v>
+        <v>227</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>79</v>
+        <v>178</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>79</v>
+        <v>228</v>
       </c>
     </row>
-    <row r="24" hidden="true">
+    <row r="24">
       <c r="A24" t="s" s="2">
-        <v>247</v>
+        <v>229</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>248</v>
+        <v>229</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
-        <v>79</v>
+        <v>230</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="G24" t="s" s="2">
         <v>87</v>
       </c>
       <c r="H24" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="I24" t="s" s="2">
         <v>79</v>
@@ -4069,16 +4172,16 @@
         <v>88</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>249</v>
+        <v>107</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>250</v>
+        <v>231</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>251</v>
+        <v>232</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>252</v>
+        <v>233</v>
       </c>
       <c r="O24" s="2"/>
       <c r="P24" t="s" s="2">
@@ -4104,13 +4207,13 @@
         <v>79</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>79</v>
+        <v>158</v>
       </c>
       <c r="Y24" t="s" s="2">
-        <v>79</v>
+        <v>234</v>
       </c>
       <c r="Z24" t="s" s="2">
-        <v>79</v>
+        <v>235</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>79</v>
@@ -4128,7 +4231,7 @@
         <v>79</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>253</v>
+        <v>229</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>77</v>
@@ -4137,41 +4240,41 @@
         <v>87</v>
       </c>
       <c r="AI24" t="s" s="2">
-        <v>254</v>
+        <v>79</v>
       </c>
       <c r="AJ24" t="s" s="2">
         <v>99</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>79</v>
+        <v>237</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>256</v>
+        <v>238</v>
       </c>
     </row>
-    <row r="25" hidden="true">
+    <row r="25">
       <c r="A25" t="s" s="2">
-        <v>257</v>
+        <v>239</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>258</v>
+        <v>239</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>79</v>
+        <v>240</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G25" t="s" s="2">
         <v>87</v>
       </c>
       <c r="H25" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="I25" t="s" s="2">
         <v>79</v>
@@ -4180,24 +4283,22 @@
         <v>88</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>249</v>
+        <v>154</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>259</v>
+        <v>241</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>260</v>
+        <v>242</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>261</v>
+        <v>243</v>
       </c>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="Q25" t="s" s="2">
-        <v>262</v>
-      </c>
+      <c r="Q25" s="2"/>
       <c r="R25" t="s" s="2">
         <v>79</v>
       </c>
@@ -4217,13 +4318,11 @@
         <v>79</v>
       </c>
       <c r="X25" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y25" t="s" s="2">
-        <v>79</v>
-      </c>
+        <v>244</v>
+      </c>
+      <c r="Y25" s="2"/>
       <c r="Z25" t="s" s="2">
-        <v>79</v>
+        <v>245</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>79</v>
@@ -4241,7 +4340,7 @@
         <v>79</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>263</v>
+        <v>239</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>77</v>
@@ -4250,56 +4349,56 @@
         <v>87</v>
       </c>
       <c r="AI25" t="s" s="2">
-        <v>254</v>
+        <v>79</v>
       </c>
       <c r="AJ25" t="s" s="2">
         <v>99</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>264</v>
+        <v>246</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>79</v>
+        <v>247</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>265</v>
+        <v>248</v>
       </c>
     </row>
-    <row r="26" hidden="true">
+    <row r="26">
       <c r="A26" t="s" s="2">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
-        <v>79</v>
+        <v>250</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G26" t="s" s="2">
         <v>87</v>
       </c>
       <c r="H26" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="I26" t="s" s="2">
         <v>79</v>
       </c>
       <c r="J26" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>267</v>
+        <v>252</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>268</v>
+        <v>253</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
@@ -4350,10 +4449,10 @@
         <v>79</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="AG26" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="AH26" t="s" s="2">
         <v>87</v>
@@ -4365,25 +4464,25 @@
         <v>99</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>269</v>
+        <v>254</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>270</v>
+        <v>255</v>
       </c>
       <c r="AM26" t="s" s="2">
-        <v>271</v>
+        <v>256</v>
       </c>
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>272</v>
+        <v>257</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>272</v>
+        <v>257</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>273</v>
+        <v>79</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
@@ -4402,13 +4501,13 @@
         <v>79</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>274</v>
+        <v>258</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -4459,7 +4558,7 @@
         <v>79</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>272</v>
+        <v>257</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>77</v>
@@ -4474,10 +4573,10 @@
         <v>99</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>277</v>
+        <v>261</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>278</v>
+        <v>262</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>79</v>
@@ -4485,14 +4584,14 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>279</v>
+        <v>263</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>279</v>
+        <v>263</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
-        <v>280</v>
+        <v>79</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
@@ -4502,26 +4601,24 @@
         <v>87</v>
       </c>
       <c r="H28" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="I28" t="s" s="2">
         <v>79</v>
       </c>
       <c r="J28" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>281</v>
+        <v>264</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>282</v>
+        <v>265</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>283</v>
-      </c>
-      <c r="N28" t="s" s="2">
-        <v>284</v>
-      </c>
+        <v>266</v>
+      </c>
+      <c r="N28" s="2"/>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>79</v>
@@ -4558,19 +4655,17 @@
         <v>79</v>
       </c>
       <c r="AB28" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC28" t="s" s="2">
-        <v>79</v>
-      </c>
+        <v>267</v>
+      </c>
+      <c r="AC28" s="2"/>
       <c r="AD28" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE28" t="s" s="2">
-        <v>79</v>
+        <v>189</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>279</v>
+        <v>263</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>77</v>
@@ -4585,23 +4680,25 @@
         <v>99</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>285</v>
+        <v>268</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>286</v>
+        <v>269</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>287</v>
+        <v>79</v>
       </c>
     </row>
-    <row r="29" hidden="true">
+    <row r="29">
       <c r="A29" t="s" s="2">
-        <v>288</v>
+        <v>270</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>288</v>
-      </c>
-      <c r="C29" s="2"/>
+        <v>263</v>
+      </c>
+      <c r="C29" t="s" s="2">
+        <v>271</v>
+      </c>
       <c r="D29" t="s" s="2">
         <v>79</v>
       </c>
@@ -4613,7 +4710,7 @@
         <v>87</v>
       </c>
       <c r="H29" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="I29" t="s" s="2">
         <v>79</v>
@@ -4622,17 +4719,15 @@
         <v>79</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>249</v>
+        <v>272</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>289</v>
+        <v>273</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>290</v>
-      </c>
-      <c r="N29" t="s" s="2">
-        <v>291</v>
-      </c>
+        <v>266</v>
+      </c>
+      <c r="N29" s="2"/>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
         <v>79</v>
@@ -4681,7 +4776,7 @@
         <v>79</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>288</v>
+        <v>263</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>77</v>
@@ -4696,10 +4791,10 @@
         <v>99</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>292</v>
+        <v>268</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>79</v>
+        <v>269</v>
       </c>
       <c r="AM29" t="s" s="2">
         <v>79</v>
@@ -4707,10 +4802,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>293</v>
+        <v>274</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>293</v>
+        <v>275</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4721,7 +4816,7 @@
         <v>77</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>79</v>
@@ -4733,17 +4828,15 @@
         <v>79</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>294</v>
+        <v>181</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>295</v>
+        <v>200</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>296</v>
-      </c>
-      <c r="N30" t="s" s="2">
-        <v>297</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>79</v>
@@ -4792,22 +4885,22 @@
         <v>79</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>293</v>
+        <v>184</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH30" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AI30" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>298</v>
+        <v>202</v>
       </c>
       <c r="AL30" t="s" s="2">
         <v>79</v>
@@ -4816,16 +4909,16 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>299</v>
+        <v>276</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>79</v>
+        <v>132</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
@@ -4835,7 +4928,7 @@
         <v>78</v>
       </c>
       <c r="H31" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="I31" t="s" s="2">
         <v>79</v>
@@ -4844,15 +4937,17 @@
         <v>79</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>300</v>
+        <v>133</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>301</v>
+        <v>134</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>302</v>
-      </c>
-      <c r="N31" s="2"/>
+        <v>278</v>
+      </c>
+      <c r="N31" t="s" s="2">
+        <v>136</v>
+      </c>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
         <v>79</v>
@@ -4889,19 +4984,19 @@
         <v>79</v>
       </c>
       <c r="AB31" t="s" s="2">
-        <v>79</v>
+        <v>188</v>
       </c>
       <c r="AC31" t="s" s="2">
-        <v>79</v>
+        <v>205</v>
       </c>
       <c r="AD31" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE31" t="s" s="2">
-        <v>79</v>
+        <v>189</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>299</v>
+        <v>190</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>77</v>
@@ -4913,10 +5008,10 @@
         <v>79</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>99</v>
+        <v>138</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>303</v>
+        <v>202</v>
       </c>
       <c r="AL31" t="s" s="2">
         <v>79</v>
@@ -4927,10 +5022,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>304</v>
+        <v>279</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>304</v>
+        <v>280</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4938,7 +5033,7 @@
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G32" t="s" s="2">
         <v>87</v>
@@ -4950,18 +5045,20 @@
         <v>79</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>236</v>
+        <v>281</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>237</v>
+        <v>282</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>238</v>
-      </c>
-      <c r="N32" s="2"/>
+        <v>283</v>
+      </c>
+      <c r="N32" t="s" s="2">
+        <v>284</v>
+      </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
         <v>79</v>
@@ -5010,7 +5107,7 @@
         <v>79</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>239</v>
+        <v>285</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>77</v>
@@ -5019,38 +5116,38 @@
         <v>87</v>
       </c>
       <c r="AI32" t="s" s="2">
-        <v>79</v>
+        <v>286</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>240</v>
+        <v>287</v>
       </c>
       <c r="AL32" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM32" t="s" s="2">
-        <v>79</v>
+        <v>288</v>
       </c>
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>305</v>
+        <v>289</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>305</v>
+        <v>290</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>132</v>
+        <v>79</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>79</v>
@@ -5059,25 +5156,27 @@
         <v>79</v>
       </c>
       <c r="J33" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>133</v>
+        <v>281</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>134</v>
+        <v>291</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>243</v>
+        <v>292</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>136</v>
+        <v>293</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="Q33" s="2"/>
+      <c r="Q33" t="s" s="2">
+        <v>294</v>
+      </c>
       <c r="R33" t="s" s="2">
         <v>79</v>
       </c>
@@ -5121,72 +5220,68 @@
         <v>79</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>246</v>
+        <v>295</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AI33" t="s" s="2">
-        <v>79</v>
+        <v>286</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>138</v>
+        <v>99</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>240</v>
+        <v>296</v>
       </c>
       <c r="AL33" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>79</v>
+        <v>297</v>
       </c>
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>307</v>
+        <v>79</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H34" t="s" s="2">
         <v>79</v>
       </c>
       <c r="I34" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>133</v>
+        <v>281</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>308</v>
+        <v>299</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>309</v>
-      </c>
-      <c r="N34" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="O34" t="s" s="2">
-        <v>142</v>
-      </c>
+        <v>300</v>
+      </c>
+      <c r="N34" s="2"/>
+      <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>79</v>
       </c>
@@ -5234,40 +5329,40 @@
         <v>79</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH34" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AI34" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>138</v>
+        <v>99</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>130</v>
+        <v>301</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>79</v>
+        <v>302</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>79</v>
+        <v>303</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
-        <v>79</v>
+        <v>305</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
@@ -5277,7 +5372,7 @@
         <v>87</v>
       </c>
       <c r="H35" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="I35" t="s" s="2">
         <v>79</v>
@@ -5286,17 +5381,15 @@
         <v>79</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>154</v>
+        <v>306</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>313</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>314</v>
-      </c>
+        <v>308</v>
+      </c>
+      <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>79</v>
@@ -5321,11 +5414,13 @@
         <v>79</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="Y35" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="Y35" t="s" s="2">
+        <v>79</v>
+      </c>
       <c r="Z35" t="s" s="2">
-        <v>315</v>
+        <v>79</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>79</v>
@@ -5343,7 +5438,7 @@
         <v>79</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>77</v>
@@ -5358,53 +5453,53 @@
         <v>99</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>79</v>
+        <v>310</v>
       </c>
       <c r="AM35" t="s" s="2">
         <v>79</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H36" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I36" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J36" t="s" s="2">
         <v>88</v>
       </c>
-      <c r="I36" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J36" t="s" s="2">
-        <v>79</v>
-      </c>
       <c r="K36" t="s" s="2">
-        <v>154</v>
+        <v>313</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
@@ -5430,13 +5525,13 @@
         <v>79</v>
       </c>
       <c r="X36" t="s" s="2">
-        <v>322</v>
+        <v>79</v>
       </c>
       <c r="Y36" t="s" s="2">
-        <v>323</v>
+        <v>79</v>
       </c>
       <c r="Z36" t="s" s="2">
-        <v>324</v>
+        <v>79</v>
       </c>
       <c r="AA36" t="s" s="2">
         <v>79</v>
@@ -5454,13 +5549,13 @@
         <v>79</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="AG36" t="s" s="2">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>79</v>
@@ -5469,25 +5564,25 @@
         <v>99</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>176</v>
+        <v>317</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>79</v>
+        <v>318</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>327</v>
+        <v>79</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
@@ -5506,16 +5601,16 @@
         <v>79</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>236</v>
+        <v>281</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -5565,7 +5660,7 @@
         <v>79</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>77</v>
@@ -5580,7 +5675,7 @@
         <v>99</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>79</v>
@@ -5589,12 +5684,12 @@
         <v>79</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5605,10 +5700,10 @@
         <v>77</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H38" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="I38" t="s" s="2">
         <v>79</v>
@@ -5617,15 +5712,17 @@
         <v>79</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>249</v>
+        <v>326</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="N38" s="2"/>
+        <v>328</v>
+      </c>
+      <c r="N38" t="s" s="2">
+        <v>329</v>
+      </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
         <v>79</v>
@@ -5674,13 +5771,13 @@
         <v>79</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI38" t="s" s="2">
         <v>79</v>
@@ -5689,21 +5786,21 @@
         <v>99</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>228</v>
+        <v>330</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>335</v>
+        <v>79</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5714,7 +5811,7 @@
         <v>77</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>88</v>
@@ -5726,17 +5823,15 @@
         <v>79</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>107</v>
+        <v>332</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>338</v>
-      </c>
-      <c r="N39" t="s" s="2">
-        <v>339</v>
-      </c>
+        <v>334</v>
+      </c>
+      <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>79</v>
@@ -5761,13 +5856,13 @@
         <v>79</v>
       </c>
       <c r="X39" t="s" s="2">
-        <v>158</v>
+        <v>79</v>
       </c>
       <c r="Y39" t="s" s="2">
-        <v>340</v>
+        <v>79</v>
       </c>
       <c r="Z39" t="s" s="2">
-        <v>341</v>
+        <v>79</v>
       </c>
       <c r="AA39" t="s" s="2">
         <v>79</v>
@@ -5785,13 +5880,13 @@
         <v>79</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH39" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI39" t="s" s="2">
         <v>79</v>
@@ -5800,7 +5895,7 @@
         <v>99</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>195</v>
+        <v>335</v>
       </c>
       <c r="AL39" t="s" s="2">
         <v>79</v>
@@ -5811,10 +5906,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5837,17 +5932,15 @@
         <v>79</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>154</v>
+        <v>181</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>343</v>
+        <v>200</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>344</v>
-      </c>
-      <c r="N40" t="s" s="2">
-        <v>345</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="N40" s="2"/>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>79</v>
@@ -5872,13 +5965,13 @@
         <v>79</v>
       </c>
       <c r="X40" t="s" s="2">
-        <v>322</v>
+        <v>79</v>
       </c>
       <c r="Y40" t="s" s="2">
-        <v>346</v>
+        <v>79</v>
       </c>
       <c r="Z40" t="s" s="2">
-        <v>347</v>
+        <v>79</v>
       </c>
       <c r="AA40" t="s" s="2">
         <v>79</v>
@@ -5896,7 +5989,7 @@
         <v>79</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>342</v>
+        <v>184</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>77</v>
@@ -5908,10 +6001,10 @@
         <v>79</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>348</v>
+        <v>202</v>
       </c>
       <c r="AL40" t="s" s="2">
         <v>79</v>
@@ -5920,16 +6013,16 @@
         <v>79</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
-        <v>79</v>
+        <v>132</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
@@ -5939,7 +6032,7 @@
         <v>78</v>
       </c>
       <c r="H41" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="I41" t="s" s="2">
         <v>79</v>
@@ -5948,16 +6041,16 @@
         <v>79</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>294</v>
+        <v>133</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>350</v>
+        <v>134</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>351</v>
+        <v>278</v>
       </c>
       <c r="N41" t="s" s="2">
-        <v>352</v>
+        <v>136</v>
       </c>
       <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
@@ -6007,7 +6100,7 @@
         <v>79</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>349</v>
+        <v>190</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>77</v>
@@ -6019,20 +6112,906 @@
         <v>79</v>
       </c>
       <c r="AJ41" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="AK41" t="s" s="2">
+        <v>202</v>
+      </c>
+      <c r="AL41" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM41" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="42" hidden="true">
+      <c r="A42" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="B42" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="C42" s="2"/>
+      <c r="D42" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="E42" s="2"/>
+      <c r="F42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G42" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I42" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="J42" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="K42" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="L42" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="M42" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="N42" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="O42" t="s" s="2">
+        <v>142</v>
+      </c>
+      <c r="P42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q42" s="2"/>
+      <c r="R42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Y42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF42" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="AG42" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH42" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ42" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="AK42" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="AL42" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM42" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="B43" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="E43" s="2"/>
+      <c r="F43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G43" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H43" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="I43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="K43" t="s" s="2">
+        <v>154</v>
+      </c>
+      <c r="L43" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="M43" t="s" s="2">
+        <v>345</v>
+      </c>
+      <c r="N43" t="s" s="2">
+        <v>346</v>
+      </c>
+      <c r="O43" s="2"/>
+      <c r="P43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q43" s="2"/>
+      <c r="R43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X43" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="Y43" s="2"/>
+      <c r="Z43" t="s" s="2">
+        <v>347</v>
+      </c>
+      <c r="AA43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF43" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="AG43" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH43" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ43" t="s" s="2">
         <v>99</v>
       </c>
-      <c r="AK41" t="s" s="2">
-        <v>298</v>
-      </c>
-      <c r="AL41" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM41" t="s" s="2">
+      <c r="AK43" t="s" s="2">
+        <v>348</v>
+      </c>
+      <c r="AL43" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM43" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="B44" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="E44" s="2"/>
+      <c r="F44" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="G44" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H44" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="I44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="K44" t="s" s="2">
+        <v>154</v>
+      </c>
+      <c r="L44" t="s" s="2">
+        <v>351</v>
+      </c>
+      <c r="M44" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="N44" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="O44" s="2"/>
+      <c r="P44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q44" s="2"/>
+      <c r="R44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X44" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="Y44" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="Z44" t="s" s="2">
+        <v>356</v>
+      </c>
+      <c r="AA44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF44" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="AG44" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AH44" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ44" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK44" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AL44" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM44" t="s" s="2">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="45" hidden="true">
+      <c r="A45" t="s" s="2">
+        <v>358</v>
+      </c>
+      <c r="B45" t="s" s="2">
+        <v>358</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" t="s" s="2">
+        <v>359</v>
+      </c>
+      <c r="E45" s="2"/>
+      <c r="F45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G45" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="K45" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="L45" t="s" s="2">
+        <v>360</v>
+      </c>
+      <c r="M45" t="s" s="2">
+        <v>361</v>
+      </c>
+      <c r="N45" t="s" s="2">
+        <v>362</v>
+      </c>
+      <c r="O45" s="2"/>
+      <c r="P45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q45" s="2"/>
+      <c r="R45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Y45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF45" t="s" s="2">
+        <v>358</v>
+      </c>
+      <c r="AG45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH45" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ45" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK45" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="AL45" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM45" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="B46" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="C46" s="2"/>
+      <c r="D46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="E46" s="2"/>
+      <c r="F46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G46" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H46" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="I46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="K46" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="L46" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="M46" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="N46" s="2"/>
+      <c r="O46" s="2"/>
+      <c r="P46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q46" s="2"/>
+      <c r="R46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Y46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF46" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="AG46" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH46" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ46" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK46" t="s" s="2">
+        <v>268</v>
+      </c>
+      <c r="AL46" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM46" t="s" s="2">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s" s="2">
+        <v>368</v>
+      </c>
+      <c r="B47" t="s" s="2">
+        <v>368</v>
+      </c>
+      <c r="C47" s="2"/>
+      <c r="D47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="E47" s="2"/>
+      <c r="F47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G47" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H47" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="I47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="K47" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="L47" t="s" s="2">
+        <v>369</v>
+      </c>
+      <c r="M47" t="s" s="2">
+        <v>370</v>
+      </c>
+      <c r="N47" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="O47" s="2"/>
+      <c r="P47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q47" s="2"/>
+      <c r="R47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X47" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="Y47" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="Z47" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="AA47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF47" t="s" s="2">
+        <v>368</v>
+      </c>
+      <c r="AG47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH47" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ47" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK47" t="s" s="2">
+        <v>236</v>
+      </c>
+      <c r="AL47" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM47" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="48" hidden="true">
+      <c r="A48" t="s" s="2">
+        <v>374</v>
+      </c>
+      <c r="B48" t="s" s="2">
+        <v>374</v>
+      </c>
+      <c r="C48" s="2"/>
+      <c r="D48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="E48" s="2"/>
+      <c r="F48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G48" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="K48" t="s" s="2">
+        <v>154</v>
+      </c>
+      <c r="L48" t="s" s="2">
+        <v>375</v>
+      </c>
+      <c r="M48" t="s" s="2">
+        <v>376</v>
+      </c>
+      <c r="N48" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="O48" s="2"/>
+      <c r="P48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q48" s="2"/>
+      <c r="R48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X48" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="Y48" t="s" s="2">
+        <v>378</v>
+      </c>
+      <c r="Z48" t="s" s="2">
+        <v>379</v>
+      </c>
+      <c r="AA48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF48" t="s" s="2">
+        <v>374</v>
+      </c>
+      <c r="AG48" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH48" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ48" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK48" t="s" s="2">
+        <v>380</v>
+      </c>
+      <c r="AL48" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM48" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s" s="2">
+        <v>381</v>
+      </c>
+      <c r="B49" t="s" s="2">
+        <v>381</v>
+      </c>
+      <c r="C49" s="2"/>
+      <c r="D49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="E49" s="2"/>
+      <c r="F49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G49" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H49" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="I49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="K49" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="L49" t="s" s="2">
+        <v>382</v>
+      </c>
+      <c r="M49" t="s" s="2">
+        <v>383</v>
+      </c>
+      <c r="N49" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="O49" s="2"/>
+      <c r="P49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q49" s="2"/>
+      <c r="R49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Y49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF49" t="s" s="2">
+        <v>381</v>
+      </c>
+      <c r="AG49" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH49" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ49" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK49" t="s" s="2">
+        <v>330</v>
+      </c>
+      <c r="AL49" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AM49" t="s" s="2">
         <v>79</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AM41">
+  <autoFilter ref="A1:AM49">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -6042,7 +7021,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI40">
+  <conditionalFormatting sqref="A2:AI48">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>